<commit_message>
feat: accuracy based validation with k
</commit_message>
<xml_diff>
--- a/validation/validation.xlsx
+++ b/validation/validation.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,40 +434,50 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>distancia</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>qtd_manifold</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>qtd_skid</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>lamina</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>cabo_elet</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>manifold</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>duto_rig</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>duto_flex</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>empresa</t>
         </is>
@@ -490,27 +500,33 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>-20.14099999999999</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-760</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>R: Petrobras; E: -1</t>
         </is>
@@ -533,27 +549,33 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-5</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-5</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>R: Petrobras; E: -1</t>
         </is>
@@ -562,43 +584,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Santos</t>
+          <t>Potiguar</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Uruguá</t>
+          <t>Biquara</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+          <t>PDI Executivo da Plataforma de Biquara (PBIQ-01)</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-170</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-21</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="n">
-        <v>-1</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>R: Petrobras; E: Petróleo Brasileiro S.A. - PETROBRAS</t>
+        <v>1</v>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: Petróleo Brasileiro S.A. - Petrobras</t>
         </is>
       </c>
     </row>
@@ -610,7 +638,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tambaú</t>
+          <t>Uruguá</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -619,72 +647,1064 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>-170</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>-21</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="n">
-        <v>-1</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>R: Petrobras; E: Petróleo Brasileiro S.A. - PETROBRAS</t>
+        <v>1</v>
+      </c>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tambaú</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Campos</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Marlim</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PDI Conceitual Parte I Petrobras Plataforma P-47 Viola</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Potiguar</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Agulha</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PDI Executivo Parcial da Plataforma de Agulha 1 (PAG-1)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Potiguar</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Biquara</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>PDI Executivo da Plataforma de Biquara (PBIQ-01)</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>-17.55</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="inlineStr">
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
+      </c>
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>R: Petrobras; E: Petróleo Brasileiro S.A. - Petrobras</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Uruguá</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tambaú</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="b">
+        <v>0</v>
+      </c>
+      <c r="F11" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Campos</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Marlim</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PDI Conceitual Parte I Petrobras Plataforma P-47 Viola</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="b">
+        <v>0</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Potiguar</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Agulha</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PDI Executivo Parcial da Plataforma de Agulha 1 (PAG-1)</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="b">
+        <v>0</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Potiguar</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Biquara</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PDI Executivo da Plataforma de Biquara (PBIQ-01)</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" t="b">
+        <v>1</v>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: Petróleo Brasileiro S.A. - Petrobras</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Uruguá</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Tambaú</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Campos</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Marlim</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PDI Conceitual Parte I Petrobras Plataforma P-47 Viola</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17" t="b">
+        <v>1</v>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" t="b">
+        <v>1</v>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Potiguar</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Agulha</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PDI Executivo Parcial da Plataforma de Agulha 1 (PAG-1)</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" t="b">
+        <v>1</v>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="b">
+        <v>1</v>
+      </c>
+      <c r="J18" t="b">
+        <v>1</v>
+      </c>
+      <c r="K18" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Potiguar</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Biquara</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PDI Executivo da Plataforma de Biquara (PBIQ-01)</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" t="b">
+        <v>1</v>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" t="b">
+        <v>0</v>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: Petróleo Brasileiro S.A. - Petrobras</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Uruguá</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" t="b">
+        <v>1</v>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tambaú</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" t="b">
+        <v>0</v>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" t="b">
+        <v>1</v>
+      </c>
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+      <c r="K21" t="b">
+        <v>1</v>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Campos</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Marlim</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>PDI Conceitual Parte I Petrobras Plataforma P-47 Viola</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" t="b">
+        <v>1</v>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="b">
+        <v>1</v>
+      </c>
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
+      <c r="K22" t="b">
+        <v>0</v>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Potiguar</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Agulha</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PDI Executivo Parcial da Plataforma de Agulha 1 (PAG-1)</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" t="b">
+        <v>1</v>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="b">
+        <v>1</v>
+      </c>
+      <c r="J23" t="b">
+        <v>1</v>
+      </c>
+      <c r="K23" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Potiguar</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Biquara</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PDI Executivo da Plataforma de Biquara (PBIQ-01)</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" t="b">
+        <v>1</v>
+      </c>
+      <c r="G24" t="b">
+        <v>1</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" t="b">
+        <v>1</v>
+      </c>
+      <c r="K24" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: Petróleo Brasileiro S.A. - Petrobras</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Uruguá</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="b">
+        <v>0</v>
+      </c>
+      <c r="F25" t="b">
+        <v>0</v>
+      </c>
+      <c r="G25" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="b">
+        <v>1</v>
+      </c>
+      <c r="J25" t="b">
+        <v>1</v>
+      </c>
+      <c r="K25" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" t="b">
+        <v>1</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Tambaú</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PDI Executivo do FPSO Cidade de Santos - Parte I</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26" t="b">
+        <v>0</v>
+      </c>
+      <c r="G26" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="b">
+        <v>1</v>
+      </c>
+      <c r="J26" t="b">
+        <v>1</v>
+      </c>
+      <c r="K26" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" t="b">
+        <v>1</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>R: Petrobras; E: -1</t>
         </is>
       </c>
     </row>

</xml_diff>